<commit_message>
Cap entry cost so a default budget can include Germany
</commit_message>
<xml_diff>
--- a/data/marketselect_countries.xlsx
+++ b/data/marketselect_countries.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="88">
   <si>
     <t xml:space="preserve">country</t>
   </si>
@@ -100,13 +100,13 @@
     <t xml:space="preserve">min spend share of market</t>
   </si>
   <si>
-    <t xml:space="preserve">Floor of 1 million USD. Not from Statista.</t>
+    <t xml:space="preserve">Entry cost is 2% of forecast revenue, floored at $2M and capped at $40M, and never above 40% of the market.</t>
   </si>
   <si>
     <t xml:space="preserve">max spend share of market</t>
   </si>
   <si>
-    <t xml:space="preserve">Cap so a large market cannot absorb the whole budget by assumption. Not from Statista.</t>
+    <t xml:space="preserve">Spend cap is 12% of forecast revenue, floored at the minimum, and capped at $80M so one country cannot take the whole budget.</t>
   </si>
   <si>
     <t xml:space="preserve">fixed cost share of min spend</t>
@@ -125,6 +125,30 @@
   </si>
   <si>
     <t xml:space="preserve">Added as market size falls toward the smallest country.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">min spend floor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Million USD. Stops a tiny market from being entered for cents.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">min spend cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Million USD. Stops Germany from requiring a $229M entry.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">max spend cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Million USD.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">min spend share ceiling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minimum spend cannot exceed this share of market size.</t>
   </si>
   <si>
     <t xml:space="preserve">Statista source series</t>
@@ -446,32 +470,32 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="32">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -500,6 +524,22 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -856,11 +896,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="71609230"/>
-        <c:axId val="33981032"/>
+        <c:axId val="49916017"/>
+        <c:axId val="52035315"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="71609230"/>
+        <c:axId val="49916017"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -892,7 +932,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="33981032"/>
+        <c:crossAx val="52035315"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -900,7 +940,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="33981032"/>
+        <c:axId val="52035315"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -966,7 +1006,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="71609230"/>
+        <c:crossAx val="49916017"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1013,9 +1053,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>1263240</xdr:colOff>
+      <xdr:colOff>1262880</xdr:colOff>
       <xdr:row>30</xdr:row>
-      <xdr:rowOff>21960</xdr:rowOff>
+      <xdr:rowOff>21600</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1024,7 +1064,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="3067200"/>
-        <a:ext cx="6479280" cy="2879280"/>
+        <a:ext cx="6478920" cy="2878920"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1045,377 +1085,377 @@
   <dimension ref="A1:I10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="2" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="2" style="1" width="22"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="str">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="str">
         <f aca="false">calc!A5</f>
         <v>United Kingdom</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="3" t="str">
         <f aca="false">calc!B5</f>
         <v>Europe</v>
       </c>
-      <c r="C2" s="3" t="n">
+      <c r="C2" s="4" t="n">
         <f aca="false">calc!C5</f>
         <v>811.657</v>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="D2" s="5" t="n">
         <f aca="false">calc!D5</f>
         <v>0.254197538609248</v>
       </c>
-      <c r="E2" s="5" t="n">
+      <c r="E2" s="6" t="n">
         <f aca="false">calc!E5</f>
         <v>0.5</v>
       </c>
-      <c r="F2" s="3" t="n">
+      <c r="F2" s="4" t="n">
         <f aca="false">calc!F5</f>
+        <v>4.058285</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <f aca="false">calc!G5</f>
         <v>16.23314</v>
       </c>
-      <c r="G2" s="3" t="n">
-        <f aca="false">calc!G5</f>
-        <v>64.93256</v>
-      </c>
-      <c r="H2" s="3" t="n">
+      <c r="H2" s="4" t="n">
         <f aca="false">calc!H5</f>
-        <v>284.07995</v>
-      </c>
-      <c r="I2" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="I2" s="6" t="n">
         <f aca="false">calc!I5</f>
         <v>0.58651804314696</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="str">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="str">
         <f aca="false">calc!A6</f>
         <v>Norway</v>
       </c>
-      <c r="B3" s="2" t="str">
+      <c r="B3" s="3" t="str">
         <f aca="false">calc!B6</f>
         <v>Europe</v>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="C3" s="4" t="n">
         <f aca="false">calc!C6</f>
         <v>324.3</v>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D3" s="5" t="n">
         <f aca="false">calc!D6</f>
         <v>0.198546637333201</v>
       </c>
-      <c r="E3" s="5" t="n">
+      <c r="E3" s="6" t="n">
         <f aca="false">calc!E6</f>
         <v>0.5</v>
       </c>
-      <c r="F3" s="3" t="n">
+      <c r="F3" s="4" t="n">
         <f aca="false">calc!F6</f>
+        <v>1.6215</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <f aca="false">calc!G6</f>
         <v>6.486</v>
       </c>
-      <c r="G3" s="3" t="n">
-        <f aca="false">calc!G6</f>
-        <v>25.944</v>
-      </c>
-      <c r="H3" s="3" t="n">
+      <c r="H3" s="4" t="n">
         <f aca="false">calc!H6</f>
-        <v>113.505</v>
-      </c>
-      <c r="I3" s="5" t="n">
+        <v>38.916</v>
+      </c>
+      <c r="I3" s="6" t="n">
         <f aca="false">calc!I6</f>
         <v>0.654657942200411</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="str">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="str">
         <f aca="false">calc!A7</f>
         <v>Spain</v>
       </c>
-      <c r="B4" s="2" t="str">
+      <c r="B4" s="3" t="str">
         <f aca="false">calc!B7</f>
         <v>Europe</v>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="C4" s="4" t="n">
         <f aca="false">calc!C7</f>
         <v>113.94</v>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" s="5" t="n">
         <f aca="false">calc!D7</f>
         <v>0.409575564718173</v>
       </c>
-      <c r="E4" s="5" t="n">
+      <c r="E4" s="6" t="n">
         <f aca="false">calc!E7</f>
         <v>0.5</v>
       </c>
-      <c r="F4" s="3" t="n">
+      <c r="F4" s="4" t="n">
         <f aca="false">calc!F7</f>
+        <v>0.5697</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <f aca="false">calc!G7</f>
         <v>2.2788</v>
       </c>
-      <c r="G4" s="3" t="n">
-        <f aca="false">calc!G7</f>
-        <v>9.1152</v>
-      </c>
-      <c r="H4" s="3" t="n">
+      <c r="H4" s="4" t="n">
         <f aca="false">calc!H7</f>
-        <v>39.879</v>
-      </c>
-      <c r="I4" s="5" t="n">
+        <v>13.6728</v>
+      </c>
+      <c r="I4" s="6" t="n">
         <f aca="false">calc!I7</f>
         <v>0.68406946017365</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="str">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="str">
         <f aca="false">calc!A8</f>
         <v>Finland</v>
       </c>
-      <c r="B5" s="2" t="str">
+      <c r="B5" s="3" t="str">
         <f aca="false">calc!B8</f>
         <v>Europe</v>
       </c>
-      <c r="C5" s="3" t="n">
+      <c r="C5" s="4" t="n">
         <f aca="false">calc!C8</f>
         <v>93.258</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="5" t="n">
         <f aca="false">calc!D8</f>
         <v>0.352294476664658</v>
       </c>
-      <c r="E5" s="5" t="n">
+      <c r="E5" s="6" t="n">
         <f aca="false">calc!E8</f>
         <v>0.5</v>
       </c>
-      <c r="F5" s="3" t="n">
+      <c r="F5" s="4" t="n">
         <f aca="false">calc!F8</f>
-        <v>1.86516</v>
-      </c>
-      <c r="G5" s="3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G5" s="4" t="n">
         <f aca="false">calc!G8</f>
-        <v>7.46064</v>
-      </c>
-      <c r="H5" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H5" s="4" t="n">
         <f aca="false">calc!H8</f>
-        <v>32.6403</v>
-      </c>
-      <c r="I5" s="5" t="n">
+        <v>11.19096</v>
+      </c>
+      <c r="I5" s="6" t="n">
         <f aca="false">calc!I8</f>
         <v>0.686961117402794</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="str">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="str">
         <f aca="false">calc!A9</f>
         <v>Germany</v>
       </c>
-      <c r="B6" s="2" t="str">
+      <c r="B6" s="3" t="str">
         <f aca="false">calc!B9</f>
         <v>Europe</v>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="C6" s="4" t="n">
         <f aca="false">calc!C9</f>
         <v>2860.92</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="5" t="n">
         <f aca="false">calc!D9</f>
         <v>0.337193047356412</v>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="E6" s="6" t="n">
         <f aca="false">calc!E9</f>
         <v>0.5</v>
       </c>
-      <c r="F6" s="3" t="n">
+      <c r="F6" s="4" t="n">
         <f aca="false">calc!F9</f>
-        <v>57.2184</v>
-      </c>
-      <c r="G6" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="G6" s="4" t="n">
         <f aca="false">calc!G9</f>
-        <v>228.8736</v>
-      </c>
-      <c r="H6" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="H6" s="4" t="n">
         <f aca="false">calc!H9</f>
-        <v>1001.322</v>
-      </c>
-      <c r="I6" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="I6" s="6" t="n">
         <f aca="false">calc!I9</f>
         <v>0.3</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="str">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="str">
         <f aca="false">calc!A10</f>
         <v>Estonia</v>
       </c>
-      <c r="B7" s="2" t="str">
+      <c r="B7" s="3" t="str">
         <f aca="false">calc!B10</f>
         <v>Europe</v>
       </c>
-      <c r="C7" s="3" t="n">
+      <c r="C7" s="4" t="n">
         <f aca="false">calc!C10</f>
         <v>7.70796</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="D7" s="5" t="n">
         <f aca="false">calc!D10</f>
         <v>0.589464067941792</v>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" s="6" t="n">
         <f aca="false">calc!E10</f>
         <v>0.5</v>
       </c>
-      <c r="F7" s="3" t="n">
+      <c r="F7" s="4" t="n">
         <f aca="false">calc!F10</f>
-        <v>0.25</v>
-      </c>
-      <c r="G7" s="3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G7" s="4" t="n">
         <f aca="false">calc!G10</f>
-        <v>1</v>
-      </c>
-      <c r="H7" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" s="4" t="n">
         <f aca="false">calc!H10</f>
-        <v>2.697786</v>
-      </c>
-      <c r="I7" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I7" s="6" t="n">
         <f aca="false">calc!I10</f>
         <v>0.698922310305776</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="str">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="str">
         <f aca="false">calc!A11</f>
         <v>Latvia</v>
       </c>
-      <c r="B8" s="2" t="str">
+      <c r="B8" s="3" t="str">
         <f aca="false">calc!B11</f>
         <v>Europe</v>
       </c>
-      <c r="C8" s="3" t="n">
+      <c r="C8" s="4" t="n">
         <f aca="false">calc!C11</f>
         <v>6.9336</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="D8" s="5" t="n">
         <f aca="false">calc!D11</f>
         <v>0.59453405182357</v>
       </c>
-      <c r="E8" s="5" t="n">
+      <c r="E8" s="6" t="n">
         <f aca="false">calc!E11</f>
         <v>0.5</v>
       </c>
-      <c r="F8" s="3" t="n">
+      <c r="F8" s="4" t="n">
         <f aca="false">calc!F11</f>
-        <v>0.25</v>
-      </c>
-      <c r="G8" s="3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G8" s="4" t="n">
         <f aca="false">calc!G11</f>
-        <v>1</v>
-      </c>
-      <c r="H8" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" s="4" t="n">
         <f aca="false">calc!H11</f>
-        <v>2.42676</v>
-      </c>
-      <c r="I8" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I8" s="6" t="n">
         <f aca="false">calc!I11</f>
         <v>0.699030577576444</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="str">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="str">
         <f aca="false">calc!A12</f>
         <v>Iceland</v>
       </c>
-      <c r="B9" s="2" t="str">
+      <c r="B9" s="3" t="str">
         <f aca="false">calc!B12</f>
         <v>Europe</v>
       </c>
-      <c r="C9" s="3" t="n">
+      <c r="C9" s="4" t="n">
         <f aca="false">calc!C12</f>
         <v>21.438</v>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="D9" s="5" t="n">
         <f aca="false">calc!D12</f>
         <v>0.252969571779648</v>
       </c>
-      <c r="E9" s="5" t="n">
+      <c r="E9" s="6" t="n">
         <f aca="false">calc!E12</f>
         <v>0.5</v>
       </c>
-      <c r="F9" s="3" t="n">
+      <c r="F9" s="4" t="n">
         <f aca="false">calc!F12</f>
-        <v>0.42876</v>
-      </c>
-      <c r="G9" s="3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G9" s="4" t="n">
         <f aca="false">calc!G12</f>
-        <v>1.71504</v>
-      </c>
-      <c r="H9" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H9" s="4" t="n">
         <f aca="false">calc!H12</f>
-        <v>7.5033</v>
-      </c>
-      <c r="I9" s="5" t="n">
+        <v>2.57256</v>
+      </c>
+      <c r="I9" s="6" t="n">
         <f aca="false">calc!I12</f>
         <v>0.697002642506606</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="str">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="str">
         <f aca="false">calc!A13</f>
         <v>Denmark</v>
       </c>
-      <c r="B10" s="2" t="str">
+      <c r="B10" s="3" t="str">
         <f aca="false">calc!B13</f>
         <v>Europe</v>
       </c>
-      <c r="C10" s="3" t="n">
+      <c r="C10" s="4" t="n">
         <f aca="false">calc!C13</f>
         <v>254.988</v>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="D10" s="5" t="n">
         <f aca="false">calc!D13</f>
         <v>0.310637984773728</v>
       </c>
-      <c r="E10" s="5" t="n">
+      <c r="E10" s="6" t="n">
         <f aca="false">calc!E13</f>
         <v>0.5</v>
       </c>
-      <c r="F10" s="3" t="n">
+      <c r="F10" s="4" t="n">
         <f aca="false">calc!F13</f>
+        <v>1.27494</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <f aca="false">calc!G13</f>
         <v>5.09976</v>
       </c>
-      <c r="G10" s="3" t="n">
-        <f aca="false">calc!G13</f>
-        <v>20.39904</v>
-      </c>
-      <c r="H10" s="3" t="n">
+      <c r="H10" s="4" t="n">
         <f aca="false">calc!H13</f>
-        <v>89.2458</v>
-      </c>
-      <c r="I10" s="5" t="n">
+        <v>30.59856</v>
+      </c>
+      <c r="I10" s="6" t="n">
         <f aca="false">calc!I13</f>
         <v>0.664348810872027</v>
       </c>
@@ -1438,12 +1478,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="6" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="6" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="6" width="88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="88"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1529,7 +1569,7 @@
         <v>22</v>
       </c>
       <c r="B11" s="13" t="n">
-        <v>0.08</v>
+        <v>0.02</v>
       </c>
       <c r="C11" s="12" t="s">
         <v>23</v>
@@ -1540,7 +1580,7 @@
         <v>24</v>
       </c>
       <c r="B12" s="13" t="n">
-        <v>0.35</v>
+        <v>0.12</v>
       </c>
       <c r="C12" s="12" t="s">
         <v>25</v>
@@ -1577,6 +1617,50 @@
       </c>
       <c r="C15" s="12" t="s">
         <v>31</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="B16" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="B17" s="15" t="n">
+        <v>40</v>
+      </c>
+      <c r="C17" s="16" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18" s="15" t="n">
+        <v>80</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="B19" s="17" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C19" s="16" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -1601,27 +1685,27 @@
   <dimension ref="A1:L13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="6" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="6" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="6" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="6" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="6" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="6" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="6" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="6" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="6" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="6" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="6" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="46"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -1636,363 +1720,363 @@
       <c r="L2" s="8"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="D4" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="E4" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="F4" s="14" t="s">
-        <v>37</v>
-      </c>
-      <c r="G4" s="14" t="s">
-        <v>38</v>
-      </c>
-      <c r="H4" s="14" t="s">
-        <v>39</v>
-      </c>
-      <c r="I4" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="J4" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="K4" s="14" t="s">
+      <c r="C4" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="L4" s="14" t="s">
+      <c r="D4" s="18" t="s">
         <v>43</v>
       </c>
+      <c r="E4" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="F4" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="G4" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="H4" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="I4" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="J4" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="K4" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="L4" s="18" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="B5" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="C5" s="16" t="n">
+      <c r="A5" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="B5" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="C5" s="20" t="n">
         <v>1411503</v>
       </c>
-      <c r="D5" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="E5" s="16" t="n">
+      <c r="D5" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="E5" s="20" t="n">
         <v>2023</v>
       </c>
-      <c r="F5" s="16" t="n">
+      <c r="F5" s="20" t="n">
         <v>2029</v>
       </c>
-      <c r="G5" s="17" t="n">
+      <c r="G5" s="21" t="n">
         <v>164.2</v>
       </c>
-      <c r="H5" s="17" t="n">
+      <c r="H5" s="21" t="n">
         <v>639.1</v>
       </c>
-      <c r="I5" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="J5" s="15" t="s">
+      <c r="I5" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="J5" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="K5" s="18" t="n">
+      <c r="K5" s="22" t="n">
         <f aca="false">F5-E5</f>
         <v>6</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="15" t="s">
-        <v>47</v>
-      </c>
-      <c r="B6" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="C6" s="16" t="n">
+      <c r="A6" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="B6" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="C6" s="20" t="n">
         <v>1413409</v>
       </c>
-      <c r="D6" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="E6" s="16" t="n">
+      <c r="D6" s="19" t="s">
+        <v>56</v>
+      </c>
+      <c r="E6" s="20" t="n">
         <v>2023</v>
       </c>
-      <c r="F6" s="16" t="n">
+      <c r="F6" s="20" t="n">
         <v>2029</v>
       </c>
-      <c r="G6" s="17" t="n">
+      <c r="G6" s="21" t="n">
         <v>109.4</v>
       </c>
-      <c r="H6" s="17" t="n">
+      <c r="H6" s="21" t="n">
         <v>324.3</v>
       </c>
-      <c r="I6" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="J6" s="15" t="s">
+      <c r="I6" s="19" t="s">
+        <v>56</v>
+      </c>
+      <c r="J6" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="K6" s="18" t="n">
+      <c r="K6" s="22" t="n">
         <f aca="false">F6-E6</f>
         <v>6</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="15" t="s">
-        <v>49</v>
-      </c>
-      <c r="B7" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="C7" s="16" t="n">
+      <c r="A7" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="C7" s="20" t="n">
         <v>1441469</v>
       </c>
-      <c r="D7" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="E7" s="16" t="n">
+      <c r="D7" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="E7" s="20" t="n">
         <v>2022</v>
       </c>
-      <c r="F7" s="16" t="n">
+      <c r="F7" s="20" t="n">
         <v>2028</v>
       </c>
-      <c r="G7" s="17" t="n">
+      <c r="G7" s="21" t="n">
         <v>13.45</v>
       </c>
-      <c r="H7" s="17" t="n">
+      <c r="H7" s="21" t="n">
         <v>105.5</v>
       </c>
-      <c r="I7" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="J7" s="15" t="s">
+      <c r="I7" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="J7" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="K7" s="18" t="n">
+      <c r="K7" s="22" t="n">
         <f aca="false">F7-E7</f>
         <v>6</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="B8" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="C8" s="16" t="n">
+      <c r="A8" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="C8" s="20" t="n">
         <v>1477322</v>
       </c>
-      <c r="D8" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="E8" s="16" t="n">
+      <c r="D8" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="E8" s="20" t="n">
         <v>2023</v>
       </c>
-      <c r="F8" s="16" t="n">
+      <c r="F8" s="20" t="n">
         <v>2029</v>
       </c>
-      <c r="G8" s="17" t="n">
+      <c r="G8" s="21" t="n">
         <v>14.12</v>
       </c>
-      <c r="H8" s="17" t="n">
+      <c r="H8" s="21" t="n">
         <v>86.35</v>
       </c>
-      <c r="I8" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="J8" s="15" t="s">
+      <c r="I8" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="J8" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="K8" s="18" t="n">
+      <c r="K8" s="22" t="n">
         <f aca="false">F8-E8</f>
         <v>6</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="15" t="s">
-        <v>52</v>
-      </c>
-      <c r="B9" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="C9" s="16" t="n">
+      <c r="A9" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="C9" s="20" t="n">
         <v>1484167</v>
       </c>
-      <c r="D9" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="E9" s="16" t="n">
+      <c r="D9" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="E9" s="20" t="n">
         <v>2023</v>
       </c>
-      <c r="F9" s="16" t="n">
+      <c r="F9" s="20" t="n">
         <v>2028</v>
       </c>
-      <c r="G9" s="17" t="n">
+      <c r="G9" s="21" t="n">
         <v>619.6</v>
       </c>
-      <c r="H9" s="17" t="n">
+      <c r="H9" s="21" t="n">
         <v>2649</v>
       </c>
-      <c r="I9" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="J9" s="15" t="s">
+      <c r="I9" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="J9" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="K9" s="18" t="n">
+      <c r="K9" s="22" t="n">
         <f aca="false">F9-E9</f>
         <v>5</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="15" t="s">
+      <c r="A10" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="B10" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="C10" s="16" t="n">
+      <c r="C10" s="20" t="n">
         <v>1499736</v>
       </c>
-      <c r="D10" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="E10" s="16" t="n">
+      <c r="D10" s="19" t="s">
+        <v>62</v>
+      </c>
+      <c r="E10" s="20" t="n">
         <v>2023</v>
       </c>
-      <c r="F10" s="16" t="n">
+      <c r="F10" s="20" t="n">
         <v>2029</v>
       </c>
-      <c r="G10" s="17" t="n">
+      <c r="G10" s="21" t="n">
         <v>0.4426</v>
       </c>
-      <c r="H10" s="17" t="n">
+      <c r="H10" s="21" t="n">
         <v>7.137</v>
       </c>
-      <c r="I10" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="J10" s="15" t="s">
+      <c r="I10" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="J10" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="K10" s="18" t="n">
+      <c r="K10" s="22" t="n">
         <f aca="false">F10-E10</f>
         <v>6</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="B11" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="C11" s="16" t="n">
+      <c r="A11" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="B11" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="C11" s="20" t="n">
         <v>1499740</v>
       </c>
-      <c r="D11" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="E11" s="16" t="n">
+      <c r="D11" s="19" t="s">
+        <v>62</v>
+      </c>
+      <c r="E11" s="20" t="n">
         <v>2023</v>
       </c>
-      <c r="F11" s="16" t="n">
+      <c r="F11" s="20" t="n">
         <v>2029</v>
       </c>
-      <c r="G11" s="17" t="n">
+      <c r="G11" s="21" t="n">
         <v>0.3906</v>
       </c>
-      <c r="H11" s="17" t="n">
+      <c r="H11" s="21" t="n">
         <v>6.42</v>
       </c>
-      <c r="I11" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="J11" s="15" t="s">
+      <c r="I11" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="J11" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="K11" s="18" t="n">
+      <c r="K11" s="22" t="n">
         <f aca="false">F11-E11</f>
         <v>6</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="B12" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="C12" s="16" t="n">
+      <c r="A12" s="19" t="s">
+        <v>64</v>
+      </c>
+      <c r="B12" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="C12" s="20" t="n">
         <v>1553214</v>
       </c>
-      <c r="D12" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="E12" s="16" t="n">
+      <c r="D12" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="E12" s="20" t="n">
         <v>2023</v>
       </c>
-      <c r="F12" s="16" t="n">
+      <c r="F12" s="20" t="n">
         <v>2029</v>
       </c>
-      <c r="G12" s="17" t="n">
+      <c r="G12" s="21" t="n">
         <v>5.13</v>
       </c>
-      <c r="H12" s="17" t="n">
+      <c r="H12" s="21" t="n">
         <v>19.85</v>
       </c>
-      <c r="I12" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="J12" s="15" t="s">
+      <c r="I12" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="J12" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="K12" s="18" t="n">
+      <c r="K12" s="22" t="n">
         <f aca="false">F12-E12</f>
         <v>6</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="15" t="s">
-        <v>57</v>
-      </c>
-      <c r="B13" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="C13" s="16" t="n">
+      <c r="A13" s="19" t="s">
+        <v>65</v>
+      </c>
+      <c r="B13" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="C13" s="20" t="n">
         <v>1553215</v>
       </c>
-      <c r="D13" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="E13" s="16" t="n">
+      <c r="D13" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="E13" s="20" t="n">
         <v>2023</v>
       </c>
-      <c r="F13" s="16" t="n">
+      <c r="F13" s="20" t="n">
         <v>2029</v>
       </c>
-      <c r="G13" s="17" t="n">
+      <c r="G13" s="21" t="n">
         <v>46.58</v>
       </c>
-      <c r="H13" s="17" t="n">
+      <c r="H13" s="21" t="n">
         <v>236.1</v>
       </c>
-      <c r="I13" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="J13" s="15" t="s">
+      <c r="I13" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="J13" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="K13" s="18" t="n">
+      <c r="K13" s="22" t="n">
         <f aca="false">F13-E13</f>
         <v>6</v>
       </c>
@@ -2021,18 +2105,18 @@
   <dimension ref="A1:L13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="6" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="2" style="6" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="2" style="1" width="18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -2047,489 +2131,489 @@
       <c r="L2" s="8"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="C4" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="14" t="s">
+      <c r="E4" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="14" t="s">
+      <c r="G4" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="14" t="s">
+      <c r="H4" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="I4" s="14" t="s">
+      <c r="I4" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="J4" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="K4" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="L4" s="14" t="s">
-        <v>37</v>
+      <c r="J4" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="K4" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="L4" s="18" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="str">
+      <c r="A5" s="23" t="str">
         <f aca="false">source!A5</f>
         <v>United Kingdom</v>
       </c>
-      <c r="B5" s="19" t="str">
+      <c r="B5" s="23" t="str">
         <f aca="false">source!B5</f>
         <v>Europe</v>
       </c>
-      <c r="C5" s="20" t="n">
+      <c r="C5" s="24" t="n">
         <f aca="false">source!H5*IF(source!J5="EUR",assumptions!$B$5,IF(source!J5="GBP",assumptions!$B$6,assumptions!$B$7))</f>
         <v>811.657</v>
       </c>
-      <c r="D5" s="21" t="n">
+      <c r="D5" s="25" t="n">
         <f aca="false">(source!H5/source!G5)^(1/source!K5)-1</f>
         <v>0.254197538609248</v>
       </c>
-      <c r="E5" s="22" t="n">
+      <c r="E5" s="26" t="n">
         <f aca="false">assumptions!$B$10</f>
         <v>0.5</v>
       </c>
-      <c r="F5" s="20" t="n">
+      <c r="F5" s="24" t="n">
         <f aca="false">assumptions!$B$13*G5</f>
+        <v>4.058285</v>
+      </c>
+      <c r="G5" s="24" t="n">
+        <f aca="false">MIN(assumptions!$B$17,MAX(assumptions!$B$16,assumptions!$B$11*C5),assumptions!$B$19*C5)</f>
         <v>16.23314</v>
       </c>
-      <c r="G5" s="20" t="n">
-        <f aca="false">MAX(1,assumptions!$B$11*C5)</f>
-        <v>64.93256</v>
-      </c>
-      <c r="H5" s="20" t="n">
-        <f aca="false">MAX(G5,assumptions!$B$12*C5)</f>
-        <v>284.07995</v>
-      </c>
-      <c r="I5" s="22" t="n">
+      <c r="H5" s="24" t="n">
+        <f aca="false">MIN(assumptions!$B$18,MAX(G5,assumptions!$B$12*C5))</f>
+        <v>80</v>
+      </c>
+      <c r="I5" s="26" t="n">
         <f aca="false">assumptions!$B$14+assumptions!$B$15*(1-C5/MAX($C$5:$C$13))</f>
         <v>0.58651804314696</v>
       </c>
-      <c r="J5" s="23" t="n">
+      <c r="J5" s="27" t="n">
         <f aca="false">source!C5</f>
         <v>1411503</v>
       </c>
-      <c r="K5" s="23" t="n">
+      <c r="K5" s="27" t="n">
         <f aca="false">source!E5</f>
         <v>2023</v>
       </c>
-      <c r="L5" s="23" t="n">
+      <c r="L5" s="27" t="n">
         <f aca="false">source!F5</f>
         <v>2029</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19" t="str">
+      <c r="A6" s="23" t="str">
         <f aca="false">source!A6</f>
         <v>Norway</v>
       </c>
-      <c r="B6" s="19" t="str">
+      <c r="B6" s="23" t="str">
         <f aca="false">source!B6</f>
         <v>Europe</v>
       </c>
-      <c r="C6" s="20" t="n">
+      <c r="C6" s="24" t="n">
         <f aca="false">source!H6*IF(source!J6="EUR",assumptions!$B$5,IF(source!J6="GBP",assumptions!$B$6,assumptions!$B$7))</f>
         <v>324.3</v>
       </c>
-      <c r="D6" s="21" t="n">
+      <c r="D6" s="25" t="n">
         <f aca="false">(source!H6/source!G6)^(1/source!K6)-1</f>
         <v>0.198546637333201</v>
       </c>
-      <c r="E6" s="22" t="n">
+      <c r="E6" s="26" t="n">
         <f aca="false">assumptions!$B$10</f>
         <v>0.5</v>
       </c>
-      <c r="F6" s="20" t="n">
+      <c r="F6" s="24" t="n">
         <f aca="false">assumptions!$B$13*G6</f>
+        <v>1.6215</v>
+      </c>
+      <c r="G6" s="24" t="n">
+        <f aca="false">MIN(assumptions!$B$17,MAX(assumptions!$B$16,assumptions!$B$11*C6),assumptions!$B$19*C6)</f>
         <v>6.486</v>
       </c>
-      <c r="G6" s="20" t="n">
-        <f aca="false">MAX(1,assumptions!$B$11*C6)</f>
-        <v>25.944</v>
-      </c>
-      <c r="H6" s="20" t="n">
-        <f aca="false">MAX(G6,assumptions!$B$12*C6)</f>
-        <v>113.505</v>
-      </c>
-      <c r="I6" s="22" t="n">
+      <c r="H6" s="24" t="n">
+        <f aca="false">MIN(assumptions!$B$18,MAX(G6,assumptions!$B$12*C6))</f>
+        <v>38.916</v>
+      </c>
+      <c r="I6" s="26" t="n">
         <f aca="false">assumptions!$B$14+assumptions!$B$15*(1-C6/MAX($C$5:$C$13))</f>
         <v>0.654657942200411</v>
       </c>
-      <c r="J6" s="23" t="n">
+      <c r="J6" s="27" t="n">
         <f aca="false">source!C6</f>
         <v>1413409</v>
       </c>
-      <c r="K6" s="23" t="n">
+      <c r="K6" s="27" t="n">
         <f aca="false">source!E6</f>
         <v>2023</v>
       </c>
-      <c r="L6" s="23" t="n">
+      <c r="L6" s="27" t="n">
         <f aca="false">source!F6</f>
         <v>2029</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="str">
+      <c r="A7" s="23" t="str">
         <f aca="false">source!A7</f>
         <v>Spain</v>
       </c>
-      <c r="B7" s="19" t="str">
+      <c r="B7" s="23" t="str">
         <f aca="false">source!B7</f>
         <v>Europe</v>
       </c>
-      <c r="C7" s="20" t="n">
+      <c r="C7" s="24" t="n">
         <f aca="false">source!H7*IF(source!J7="EUR",assumptions!$B$5,IF(source!J7="GBP",assumptions!$B$6,assumptions!$B$7))</f>
         <v>113.94</v>
       </c>
-      <c r="D7" s="21" t="n">
+      <c r="D7" s="25" t="n">
         <f aca="false">(source!H7/source!G7)^(1/source!K7)-1</f>
         <v>0.409575564718173</v>
       </c>
-      <c r="E7" s="22" t="n">
+      <c r="E7" s="26" t="n">
         <f aca="false">assumptions!$B$10</f>
         <v>0.5</v>
       </c>
-      <c r="F7" s="20" t="n">
+      <c r="F7" s="24" t="n">
         <f aca="false">assumptions!$B$13*G7</f>
+        <v>0.5697</v>
+      </c>
+      <c r="G7" s="24" t="n">
+        <f aca="false">MIN(assumptions!$B$17,MAX(assumptions!$B$16,assumptions!$B$11*C7),assumptions!$B$19*C7)</f>
         <v>2.2788</v>
       </c>
-      <c r="G7" s="20" t="n">
-        <f aca="false">MAX(1,assumptions!$B$11*C7)</f>
-        <v>9.1152</v>
-      </c>
-      <c r="H7" s="20" t="n">
-        <f aca="false">MAX(G7,assumptions!$B$12*C7)</f>
-        <v>39.879</v>
-      </c>
-      <c r="I7" s="22" t="n">
+      <c r="H7" s="24" t="n">
+        <f aca="false">MIN(assumptions!$B$18,MAX(G7,assumptions!$B$12*C7))</f>
+        <v>13.6728</v>
+      </c>
+      <c r="I7" s="26" t="n">
         <f aca="false">assumptions!$B$14+assumptions!$B$15*(1-C7/MAX($C$5:$C$13))</f>
         <v>0.68406946017365</v>
       </c>
-      <c r="J7" s="23" t="n">
+      <c r="J7" s="27" t="n">
         <f aca="false">source!C7</f>
         <v>1441469</v>
       </c>
-      <c r="K7" s="23" t="n">
+      <c r="K7" s="27" t="n">
         <f aca="false">source!E7</f>
         <v>2022</v>
       </c>
-      <c r="L7" s="23" t="n">
+      <c r="L7" s="27" t="n">
         <f aca="false">source!F7</f>
         <v>2028</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="str">
+      <c r="A8" s="23" t="str">
         <f aca="false">source!A8</f>
         <v>Finland</v>
       </c>
-      <c r="B8" s="19" t="str">
+      <c r="B8" s="23" t="str">
         <f aca="false">source!B8</f>
         <v>Europe</v>
       </c>
-      <c r="C8" s="20" t="n">
+      <c r="C8" s="24" t="n">
         <f aca="false">source!H8*IF(source!J8="EUR",assumptions!$B$5,IF(source!J8="GBP",assumptions!$B$6,assumptions!$B$7))</f>
         <v>93.258</v>
       </c>
-      <c r="D8" s="21" t="n">
+      <c r="D8" s="25" t="n">
         <f aca="false">(source!H8/source!G8)^(1/source!K8)-1</f>
         <v>0.352294476664658</v>
       </c>
-      <c r="E8" s="22" t="n">
+      <c r="E8" s="26" t="n">
         <f aca="false">assumptions!$B$10</f>
         <v>0.5</v>
       </c>
-      <c r="F8" s="20" t="n">
+      <c r="F8" s="24" t="n">
         <f aca="false">assumptions!$B$13*G8</f>
-        <v>1.86516</v>
-      </c>
-      <c r="G8" s="20" t="n">
-        <f aca="false">MAX(1,assumptions!$B$11*C8)</f>
-        <v>7.46064</v>
-      </c>
-      <c r="H8" s="20" t="n">
-        <f aca="false">MAX(G8,assumptions!$B$12*C8)</f>
-        <v>32.6403</v>
-      </c>
-      <c r="I8" s="22" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G8" s="24" t="n">
+        <f aca="false">MIN(assumptions!$B$17,MAX(assumptions!$B$16,assumptions!$B$11*C8),assumptions!$B$19*C8)</f>
+        <v>2</v>
+      </c>
+      <c r="H8" s="24" t="n">
+        <f aca="false">MIN(assumptions!$B$18,MAX(G8,assumptions!$B$12*C8))</f>
+        <v>11.19096</v>
+      </c>
+      <c r="I8" s="26" t="n">
         <f aca="false">assumptions!$B$14+assumptions!$B$15*(1-C8/MAX($C$5:$C$13))</f>
         <v>0.686961117402794</v>
       </c>
-      <c r="J8" s="23" t="n">
+      <c r="J8" s="27" t="n">
         <f aca="false">source!C8</f>
         <v>1477322</v>
       </c>
-      <c r="K8" s="23" t="n">
+      <c r="K8" s="27" t="n">
         <f aca="false">source!E8</f>
         <v>2023</v>
       </c>
-      <c r="L8" s="23" t="n">
+      <c r="L8" s="27" t="n">
         <f aca="false">source!F8</f>
         <v>2029</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="str">
+      <c r="A9" s="23" t="str">
         <f aca="false">source!A9</f>
         <v>Germany</v>
       </c>
-      <c r="B9" s="19" t="str">
+      <c r="B9" s="23" t="str">
         <f aca="false">source!B9</f>
         <v>Europe</v>
       </c>
-      <c r="C9" s="20" t="n">
+      <c r="C9" s="24" t="n">
         <f aca="false">source!H9*IF(source!J9="EUR",assumptions!$B$5,IF(source!J9="GBP",assumptions!$B$6,assumptions!$B$7))</f>
         <v>2860.92</v>
       </c>
-      <c r="D9" s="21" t="n">
+      <c r="D9" s="25" t="n">
         <f aca="false">(source!H9/source!G9)^(1/source!K9)-1</f>
         <v>0.337193047356412</v>
       </c>
-      <c r="E9" s="22" t="n">
+      <c r="E9" s="26" t="n">
         <f aca="false">assumptions!$B$10</f>
         <v>0.5</v>
       </c>
-      <c r="F9" s="20" t="n">
+      <c r="F9" s="24" t="n">
         <f aca="false">assumptions!$B$13*G9</f>
-        <v>57.2184</v>
-      </c>
-      <c r="G9" s="20" t="n">
-        <f aca="false">MAX(1,assumptions!$B$11*C9)</f>
-        <v>228.8736</v>
-      </c>
-      <c r="H9" s="20" t="n">
-        <f aca="false">MAX(G9,assumptions!$B$12*C9)</f>
-        <v>1001.322</v>
-      </c>
-      <c r="I9" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G9" s="24" t="n">
+        <f aca="false">MIN(assumptions!$B$17,MAX(assumptions!$B$16,assumptions!$B$11*C9),assumptions!$B$19*C9)</f>
+        <v>40</v>
+      </c>
+      <c r="H9" s="24" t="n">
+        <f aca="false">MIN(assumptions!$B$18,MAX(G9,assumptions!$B$12*C9))</f>
+        <v>80</v>
+      </c>
+      <c r="I9" s="26" t="n">
         <f aca="false">assumptions!$B$14+assumptions!$B$15*(1-C9/MAX($C$5:$C$13))</f>
         <v>0.3</v>
       </c>
-      <c r="J9" s="23" t="n">
+      <c r="J9" s="27" t="n">
         <f aca="false">source!C9</f>
         <v>1484167</v>
       </c>
-      <c r="K9" s="23" t="n">
+      <c r="K9" s="27" t="n">
         <f aca="false">source!E9</f>
         <v>2023</v>
       </c>
-      <c r="L9" s="23" t="n">
+      <c r="L9" s="27" t="n">
         <f aca="false">source!F9</f>
         <v>2028</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="str">
+      <c r="A10" s="23" t="str">
         <f aca="false">source!A10</f>
         <v>Estonia</v>
       </c>
-      <c r="B10" s="19" t="str">
+      <c r="B10" s="23" t="str">
         <f aca="false">source!B10</f>
         <v>Europe</v>
       </c>
-      <c r="C10" s="20" t="n">
+      <c r="C10" s="24" t="n">
         <f aca="false">source!H10*IF(source!J10="EUR",assumptions!$B$5,IF(source!J10="GBP",assumptions!$B$6,assumptions!$B$7))</f>
         <v>7.70796</v>
       </c>
-      <c r="D10" s="21" t="n">
+      <c r="D10" s="25" t="n">
         <f aca="false">(source!H10/source!G10)^(1/source!K10)-1</f>
         <v>0.589464067941792</v>
       </c>
-      <c r="E10" s="22" t="n">
+      <c r="E10" s="26" t="n">
         <f aca="false">assumptions!$B$10</f>
         <v>0.5</v>
       </c>
-      <c r="F10" s="20" t="n">
+      <c r="F10" s="24" t="n">
         <f aca="false">assumptions!$B$13*G10</f>
-        <v>0.25</v>
-      </c>
-      <c r="G10" s="20" t="n">
-        <f aca="false">MAX(1,assumptions!$B$11*C10)</f>
-        <v>1</v>
-      </c>
-      <c r="H10" s="20" t="n">
-        <f aca="false">MAX(G10,assumptions!$B$12*C10)</f>
-        <v>2.697786</v>
-      </c>
-      <c r="I10" s="22" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G10" s="24" t="n">
+        <f aca="false">MIN(assumptions!$B$17,MAX(assumptions!$B$16,assumptions!$B$11*C10),assumptions!$B$19*C10)</f>
+        <v>2</v>
+      </c>
+      <c r="H10" s="24" t="n">
+        <f aca="false">MIN(assumptions!$B$18,MAX(G10,assumptions!$B$12*C10))</f>
+        <v>2</v>
+      </c>
+      <c r="I10" s="26" t="n">
         <f aca="false">assumptions!$B$14+assumptions!$B$15*(1-C10/MAX($C$5:$C$13))</f>
         <v>0.698922310305776</v>
       </c>
-      <c r="J10" s="23" t="n">
+      <c r="J10" s="27" t="n">
         <f aca="false">source!C10</f>
         <v>1499736</v>
       </c>
-      <c r="K10" s="23" t="n">
+      <c r="K10" s="27" t="n">
         <f aca="false">source!E10</f>
         <v>2023</v>
       </c>
-      <c r="L10" s="23" t="n">
+      <c r="L10" s="27" t="n">
         <f aca="false">source!F10</f>
         <v>2029</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19" t="str">
+      <c r="A11" s="23" t="str">
         <f aca="false">source!A11</f>
         <v>Latvia</v>
       </c>
-      <c r="B11" s="19" t="str">
+      <c r="B11" s="23" t="str">
         <f aca="false">source!B11</f>
         <v>Europe</v>
       </c>
-      <c r="C11" s="20" t="n">
+      <c r="C11" s="24" t="n">
         <f aca="false">source!H11*IF(source!J11="EUR",assumptions!$B$5,IF(source!J11="GBP",assumptions!$B$6,assumptions!$B$7))</f>
         <v>6.9336</v>
       </c>
-      <c r="D11" s="21" t="n">
+      <c r="D11" s="25" t="n">
         <f aca="false">(source!H11/source!G11)^(1/source!K11)-1</f>
         <v>0.59453405182357</v>
       </c>
-      <c r="E11" s="22" t="n">
+      <c r="E11" s="26" t="n">
         <f aca="false">assumptions!$B$10</f>
         <v>0.5</v>
       </c>
-      <c r="F11" s="20" t="n">
+      <c r="F11" s="24" t="n">
         <f aca="false">assumptions!$B$13*G11</f>
-        <v>0.25</v>
-      </c>
-      <c r="G11" s="20" t="n">
-        <f aca="false">MAX(1,assumptions!$B$11*C11)</f>
-        <v>1</v>
-      </c>
-      <c r="H11" s="20" t="n">
-        <f aca="false">MAX(G11,assumptions!$B$12*C11)</f>
-        <v>2.42676</v>
-      </c>
-      <c r="I11" s="22" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G11" s="24" t="n">
+        <f aca="false">MIN(assumptions!$B$17,MAX(assumptions!$B$16,assumptions!$B$11*C11),assumptions!$B$19*C11)</f>
+        <v>2</v>
+      </c>
+      <c r="H11" s="24" t="n">
+        <f aca="false">MIN(assumptions!$B$18,MAX(G11,assumptions!$B$12*C11))</f>
+        <v>2</v>
+      </c>
+      <c r="I11" s="26" t="n">
         <f aca="false">assumptions!$B$14+assumptions!$B$15*(1-C11/MAX($C$5:$C$13))</f>
         <v>0.699030577576444</v>
       </c>
-      <c r="J11" s="23" t="n">
+      <c r="J11" s="27" t="n">
         <f aca="false">source!C11</f>
         <v>1499740</v>
       </c>
-      <c r="K11" s="23" t="n">
+      <c r="K11" s="27" t="n">
         <f aca="false">source!E11</f>
         <v>2023</v>
       </c>
-      <c r="L11" s="23" t="n">
+      <c r="L11" s="27" t="n">
         <f aca="false">source!F11</f>
         <v>2029</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="19" t="str">
+      <c r="A12" s="23" t="str">
         <f aca="false">source!A12</f>
         <v>Iceland</v>
       </c>
-      <c r="B12" s="19" t="str">
+      <c r="B12" s="23" t="str">
         <f aca="false">source!B12</f>
         <v>Europe</v>
       </c>
-      <c r="C12" s="20" t="n">
+      <c r="C12" s="24" t="n">
         <f aca="false">source!H12*IF(source!J12="EUR",assumptions!$B$5,IF(source!J12="GBP",assumptions!$B$6,assumptions!$B$7))</f>
         <v>21.438</v>
       </c>
-      <c r="D12" s="21" t="n">
+      <c r="D12" s="25" t="n">
         <f aca="false">(source!H12/source!G12)^(1/source!K12)-1</f>
         <v>0.252969571779648</v>
       </c>
-      <c r="E12" s="22" t="n">
+      <c r="E12" s="26" t="n">
         <f aca="false">assumptions!$B$10</f>
         <v>0.5</v>
       </c>
-      <c r="F12" s="20" t="n">
+      <c r="F12" s="24" t="n">
         <f aca="false">assumptions!$B$13*G12</f>
-        <v>0.42876</v>
-      </c>
-      <c r="G12" s="20" t="n">
-        <f aca="false">MAX(1,assumptions!$B$11*C12)</f>
-        <v>1.71504</v>
-      </c>
-      <c r="H12" s="20" t="n">
-        <f aca="false">MAX(G12,assumptions!$B$12*C12)</f>
-        <v>7.5033</v>
-      </c>
-      <c r="I12" s="22" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G12" s="24" t="n">
+        <f aca="false">MIN(assumptions!$B$17,MAX(assumptions!$B$16,assumptions!$B$11*C12),assumptions!$B$19*C12)</f>
+        <v>2</v>
+      </c>
+      <c r="H12" s="24" t="n">
+        <f aca="false">MIN(assumptions!$B$18,MAX(G12,assumptions!$B$12*C12))</f>
+        <v>2.57256</v>
+      </c>
+      <c r="I12" s="26" t="n">
         <f aca="false">assumptions!$B$14+assumptions!$B$15*(1-C12/MAX($C$5:$C$13))</f>
         <v>0.697002642506606</v>
       </c>
-      <c r="J12" s="23" t="n">
+      <c r="J12" s="27" t="n">
         <f aca="false">source!C12</f>
         <v>1553214</v>
       </c>
-      <c r="K12" s="23" t="n">
+      <c r="K12" s="27" t="n">
         <f aca="false">source!E12</f>
         <v>2023</v>
       </c>
-      <c r="L12" s="23" t="n">
+      <c r="L12" s="27" t="n">
         <f aca="false">source!F12</f>
         <v>2029</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="19" t="str">
+      <c r="A13" s="23" t="str">
         <f aca="false">source!A13</f>
         <v>Denmark</v>
       </c>
-      <c r="B13" s="19" t="str">
+      <c r="B13" s="23" t="str">
         <f aca="false">source!B13</f>
         <v>Europe</v>
       </c>
-      <c r="C13" s="20" t="n">
+      <c r="C13" s="24" t="n">
         <f aca="false">source!H13*IF(source!J13="EUR",assumptions!$B$5,IF(source!J13="GBP",assumptions!$B$6,assumptions!$B$7))</f>
         <v>254.988</v>
       </c>
-      <c r="D13" s="21" t="n">
+      <c r="D13" s="25" t="n">
         <f aca="false">(source!H13/source!G13)^(1/source!K13)-1</f>
         <v>0.310637984773728</v>
       </c>
-      <c r="E13" s="22" t="n">
+      <c r="E13" s="26" t="n">
         <f aca="false">assumptions!$B$10</f>
         <v>0.5</v>
       </c>
-      <c r="F13" s="20" t="n">
+      <c r="F13" s="24" t="n">
         <f aca="false">assumptions!$B$13*G13</f>
+        <v>1.27494</v>
+      </c>
+      <c r="G13" s="24" t="n">
+        <f aca="false">MIN(assumptions!$B$17,MAX(assumptions!$B$16,assumptions!$B$11*C13),assumptions!$B$19*C13)</f>
         <v>5.09976</v>
       </c>
-      <c r="G13" s="20" t="n">
-        <f aca="false">MAX(1,assumptions!$B$11*C13)</f>
-        <v>20.39904</v>
-      </c>
-      <c r="H13" s="20" t="n">
-        <f aca="false">MAX(G13,assumptions!$B$12*C13)</f>
-        <v>89.2458</v>
-      </c>
-      <c r="I13" s="22" t="n">
+      <c r="H13" s="24" t="n">
+        <f aca="false">MIN(assumptions!$B$18,MAX(G13,assumptions!$B$12*C13))</f>
+        <v>30.59856</v>
+      </c>
+      <c r="I13" s="26" t="n">
         <f aca="false">assumptions!$B$14+assumptions!$B$15*(1-C13/MAX($C$5:$C$13))</f>
         <v>0.664348810872027</v>
       </c>
-      <c r="J13" s="23" t="n">
+      <c r="J13" s="27" t="n">
         <f aca="false">source!C13</f>
         <v>1553215</v>
       </c>
-      <c r="K13" s="23" t="n">
+      <c r="K13" s="27" t="n">
         <f aca="false">source!E13</f>
         <v>2023</v>
       </c>
-      <c r="L13" s="23" t="n">
+      <c r="L13" s="27" t="n">
         <f aca="false">source!F13</f>
         <v>2029</v>
       </c>
@@ -2558,22 +2642,22 @@
   <dimension ref="A1:G13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="6" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="6" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="6" width="78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="6" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="6" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="6" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -2583,278 +2667,278 @@
       <c r="G2" s="8"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>62</v>
-      </c>
-      <c r="D4" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="E4" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="F4" s="14" t="s">
-        <v>43</v>
-      </c>
-      <c r="G4" s="14" t="s">
-        <v>65</v>
+      <c r="B4" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="D4" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="E4" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="F4" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="G4" s="18" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="24" t="str">
+      <c r="A5" s="28" t="str">
         <f aca="false">source!A5</f>
         <v>United Kingdom</v>
       </c>
-      <c r="B5" s="25" t="n">
+      <c r="B5" s="29" t="n">
         <f aca="false">source!C5</f>
         <v>1411503</v>
       </c>
-      <c r="C5" s="26" t="s">
-        <v>66</v>
-      </c>
-      <c r="D5" s="24" t="str">
+      <c r="C5" s="30" t="s">
+        <v>74</v>
+      </c>
+      <c r="D5" s="28" t="str">
         <f aca="false">source!D5</f>
         <v>million GBP</v>
       </c>
-      <c r="E5" s="26" t="str">
+      <c r="E5" s="30" t="str">
         <f aca="false">source!E5&amp;"-"&amp;source!F5</f>
         <v>2023-2029</v>
       </c>
-      <c r="F5" s="24" t="n">
+      <c r="F5" s="28" t="n">
         <f aca="false">source!L5</f>
         <v>0</v>
       </c>
-      <c r="G5" s="27" t="s">
-        <v>67</v>
+      <c r="G5" s="31" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="24" t="str">
+      <c r="A6" s="28" t="str">
         <f aca="false">source!A6</f>
         <v>Norway</v>
       </c>
-      <c r="B6" s="25" t="n">
+      <c r="B6" s="29" t="n">
         <f aca="false">source!C6</f>
         <v>1413409</v>
       </c>
-      <c r="C6" s="26" t="s">
-        <v>68</v>
-      </c>
-      <c r="D6" s="24" t="str">
+      <c r="C6" s="30" t="s">
+        <v>76</v>
+      </c>
+      <c r="D6" s="28" t="str">
         <f aca="false">source!D6</f>
         <v>million USD</v>
       </c>
-      <c r="E6" s="26" t="str">
+      <c r="E6" s="30" t="str">
         <f aca="false">source!E6&amp;"-"&amp;source!F6</f>
         <v>2023-2029</v>
       </c>
-      <c r="F6" s="24" t="n">
+      <c r="F6" s="28" t="n">
         <f aca="false">source!L6</f>
         <v>0</v>
       </c>
-      <c r="G6" s="27" t="s">
-        <v>69</v>
+      <c r="G6" s="31" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="24" t="str">
+      <c r="A7" s="28" t="str">
         <f aca="false">source!A7</f>
         <v>Spain</v>
       </c>
-      <c r="B7" s="25" t="n">
+      <c r="B7" s="29" t="n">
         <f aca="false">source!C7</f>
         <v>1441469</v>
       </c>
-      <c r="C7" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="D7" s="24" t="str">
+      <c r="C7" s="30" t="s">
+        <v>78</v>
+      </c>
+      <c r="D7" s="28" t="str">
         <f aca="false">source!D7</f>
         <v>million EUR</v>
       </c>
-      <c r="E7" s="26" t="str">
+      <c r="E7" s="30" t="str">
         <f aca="false">source!E7&amp;"-"&amp;source!F7</f>
         <v>2022-2028</v>
       </c>
-      <c r="F7" s="24" t="n">
+      <c r="F7" s="28" t="n">
         <f aca="false">source!L7</f>
         <v>0</v>
       </c>
-      <c r="G7" s="27" t="s">
-        <v>71</v>
+      <c r="G7" s="31" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="24" t="str">
+      <c r="A8" s="28" t="str">
         <f aca="false">source!A8</f>
         <v>Finland</v>
       </c>
-      <c r="B8" s="25" t="n">
+      <c r="B8" s="29" t="n">
         <f aca="false">source!C8</f>
         <v>1477322</v>
       </c>
-      <c r="C8" s="26" t="s">
-        <v>72</v>
-      </c>
-      <c r="D8" s="24" t="str">
+      <c r="C8" s="30" t="s">
+        <v>80</v>
+      </c>
+      <c r="D8" s="28" t="str">
         <f aca="false">source!D8</f>
         <v>million EUR</v>
       </c>
-      <c r="E8" s="26" t="str">
+      <c r="E8" s="30" t="str">
         <f aca="false">source!E8&amp;"-"&amp;source!F8</f>
         <v>2023-2029</v>
       </c>
-      <c r="F8" s="24" t="n">
+      <c r="F8" s="28" t="n">
         <f aca="false">source!L8</f>
         <v>0</v>
       </c>
-      <c r="G8" s="27" t="s">
-        <v>67</v>
+      <c r="G8" s="31" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="24" t="str">
+      <c r="A9" s="28" t="str">
         <f aca="false">source!A9</f>
         <v>Germany</v>
       </c>
-      <c r="B9" s="25" t="n">
+      <c r="B9" s="29" t="n">
         <f aca="false">source!C9</f>
         <v>1484167</v>
       </c>
-      <c r="C9" s="26" t="s">
-        <v>73</v>
-      </c>
-      <c r="D9" s="24" t="str">
+      <c r="C9" s="30" t="s">
+        <v>81</v>
+      </c>
+      <c r="D9" s="28" t="str">
         <f aca="false">source!D9</f>
         <v>million EUR</v>
       </c>
-      <c r="E9" s="26" t="str">
+      <c r="E9" s="30" t="str">
         <f aca="false">source!E9&amp;"-"&amp;source!F9</f>
         <v>2023-2028</v>
       </c>
-      <c r="F9" s="24" t="n">
+      <c r="F9" s="28" t="n">
         <f aca="false">source!L9</f>
         <v>0</v>
       </c>
-      <c r="G9" s="27" t="s">
-        <v>71</v>
+      <c r="G9" s="31" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="24" t="str">
+      <c r="A10" s="28" t="str">
         <f aca="false">source!A10</f>
         <v>Estonia</v>
       </c>
-      <c r="B10" s="25" t="n">
+      <c r="B10" s="29" t="n">
         <f aca="false">source!C10</f>
         <v>1499736</v>
       </c>
-      <c r="C10" s="26" t="s">
-        <v>74</v>
-      </c>
-      <c r="D10" s="24" t="str">
+      <c r="C10" s="30" t="s">
+        <v>82</v>
+      </c>
+      <c r="D10" s="28" t="str">
         <f aca="false">source!D10</f>
         <v>thousand EUR</v>
       </c>
-      <c r="E10" s="26" t="str">
+      <c r="E10" s="30" t="str">
         <f aca="false">source!E10&amp;"-"&amp;source!F10</f>
         <v>2023-2029</v>
       </c>
-      <c r="F10" s="24" t="n">
+      <c r="F10" s="28" t="n">
         <f aca="false">source!L10</f>
         <v>0</v>
       </c>
-      <c r="G10" s="27" t="s">
-        <v>75</v>
+      <c r="G10" s="31" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="24" t="str">
+      <c r="A11" s="28" t="str">
         <f aca="false">source!A11</f>
         <v>Latvia</v>
       </c>
-      <c r="B11" s="25" t="n">
+      <c r="B11" s="29" t="n">
         <f aca="false">source!C11</f>
         <v>1499740</v>
       </c>
-      <c r="C11" s="26" t="s">
-        <v>76</v>
-      </c>
-      <c r="D11" s="24" t="str">
+      <c r="C11" s="30" t="s">
+        <v>84</v>
+      </c>
+      <c r="D11" s="28" t="str">
         <f aca="false">source!D11</f>
         <v>thousand EUR</v>
       </c>
-      <c r="E11" s="26" t="str">
+      <c r="E11" s="30" t="str">
         <f aca="false">source!E11&amp;"-"&amp;source!F11</f>
         <v>2023-2029</v>
       </c>
-      <c r="F11" s="24" t="n">
+      <c r="F11" s="28" t="n">
         <f aca="false">source!L11</f>
         <v>0</v>
       </c>
-      <c r="G11" s="27" t="s">
-        <v>75</v>
+      <c r="G11" s="31" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="24" t="str">
+      <c r="A12" s="28" t="str">
         <f aca="false">source!A12</f>
         <v>Iceland</v>
       </c>
-      <c r="B12" s="25" t="n">
+      <c r="B12" s="29" t="n">
         <f aca="false">source!C12</f>
         <v>1553214</v>
       </c>
-      <c r="C12" s="26" t="s">
-        <v>77</v>
-      </c>
-      <c r="D12" s="24" t="str">
+      <c r="C12" s="30" t="s">
+        <v>85</v>
+      </c>
+      <c r="D12" s="28" t="str">
         <f aca="false">source!D12</f>
         <v>million EUR</v>
       </c>
-      <c r="E12" s="26" t="str">
+      <c r="E12" s="30" t="str">
         <f aca="false">source!E12&amp;"-"&amp;source!F12</f>
         <v>2023-2029</v>
       </c>
-      <c r="F12" s="24" t="n">
+      <c r="F12" s="28" t="n">
         <f aca="false">source!L12</f>
         <v>0</v>
       </c>
-      <c r="G12" s="27" t="s">
-        <v>78</v>
+      <c r="G12" s="31" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="24" t="str">
+      <c r="A13" s="28" t="str">
         <f aca="false">source!A13</f>
         <v>Denmark</v>
       </c>
-      <c r="B13" s="25" t="n">
+      <c r="B13" s="29" t="n">
         <f aca="false">source!C13</f>
         <v>1553215</v>
       </c>
-      <c r="C13" s="26" t="s">
-        <v>79</v>
-      </c>
-      <c r="D13" s="24" t="str">
+      <c r="C13" s="30" t="s">
+        <v>87</v>
+      </c>
+      <c r="D13" s="28" t="str">
         <f aca="false">source!D13</f>
         <v>million EUR</v>
       </c>
-      <c r="E13" s="26" t="str">
+      <c r="E13" s="30" t="str">
         <f aca="false">source!E13&amp;"-"&amp;source!F13</f>
         <v>2023-2029</v>
       </c>
-      <c r="F13" s="24" t="n">
+      <c r="F13" s="28" t="n">
         <f aca="false">source!L13</f>
         <v>0</v>
       </c>
-      <c r="G13" s="27" t="s">
-        <v>78</v>
+      <c r="G13" s="31" t="s">
+        <v>86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>